<commit_message>
data(listing-raw): sikbom 원본양식 갱신
</commit_message>
<xml_diff>
--- a/reference/listing_sikbom.xlsx
+++ b/reference/listing_sikbom.xlsx
@@ -3769,7 +3769,7 @@
       </c>
       <c r="S27" s="7" t="inlineStr">
         <is>
-          <t>17300</t>
+          <t>19500</t>
         </is>
       </c>
       <c r="T27" s="7" t="inlineStr">
@@ -27645,7 +27645,7 @@
       </c>
       <c r="S181" s="7" t="inlineStr">
         <is>
-          <t>59300</t>
+          <t>64500</t>
         </is>
       </c>
       <c r="T181" s="7" t="inlineStr">
@@ -29361,7 +29361,7 @@
       </c>
       <c r="S192" s="7" t="inlineStr">
         <is>
-          <t>10600</t>
+          <t>11500</t>
         </is>
       </c>
       <c r="T192" s="7" t="inlineStr">
@@ -66653,7 +66653,7 @@
       </c>
       <c r="S431" s="7" t="inlineStr">
         <is>
-          <t>20300</t>
+          <t>22700</t>
         </is>
       </c>
       <c r="T431" s="7" t="inlineStr">

</xml_diff>